<commit_message>
Update Excel files and modify email template for remittance monitoring; adjust paths in scripts
</commit_message>
<xml_diff>
--- a/dados/inputs/Contatos Regionais.xlsx
+++ b/dados/inputs/Contatos Regionais.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m755247\Desktop\REPOSITORIOS\scripts\sei\script-sei-envia-monit-cronograma\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m755247\Desktop\REPOSITORIOS\scripts\sei\script-sei-envia-monit-cronograma\dados\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="dados" sheetId="3" r:id="rId1"/>
-    <sheet name="teste" sheetId="1" r:id="rId2"/>
+    <sheet name="backup" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="155">
-  <si>
-    <t>MUNICIPIO</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="162">
   <si>
     <t>ALFENAS</t>
   </si>
@@ -503,14 +500,38 @@
     <t>EMAIL_UNIDADE_REGIONAL</t>
   </si>
   <si>
-    <t>gustavo.bernardino@ipsemg.mg.gov.br</t>
+    <t>DIVINOPOLIS</t>
+  </si>
+  <si>
+    <t>ITAUNA</t>
+  </si>
+  <si>
+    <t>MANHUACU</t>
+  </si>
+  <si>
+    <t>MUNICIPIO_FFE</t>
+  </si>
+  <si>
+    <t>MUNICIPIO_DL</t>
+  </si>
+  <si>
+    <t>MURIAE</t>
+  </si>
+  <si>
+    <t>POCOS DE CALDAS</t>
+  </si>
+  <si>
+    <t>TEOFILO OTONI</t>
+  </si>
+  <si>
+    <t>UBA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -520,13 +541,6 @@
     </font>
     <font>
       <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -551,19 +565,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
+  <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -581,10 +591,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="contatos_teste" displayName="contatos_teste" ref="A1:D39" totalsRowShown="0">
-  <autoFilter ref="A1:D39"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="MUNICIPIO"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="contatos_teste245" displayName="contatos_teste245" ref="A1:E39" totalsRowShown="0">
+  <autoFilter ref="A1:E39"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="MUNICIPIO_FFE"/>
+    <tableColumn id="5" name="MUNICIPIO_DL"/>
     <tableColumn id="2" name="UNIDADE_REGIONAL_FFE"/>
     <tableColumn id="3" name="EMAIL_COORDENADOR"/>
     <tableColumn id="4" name="EMAIL_UNIDADE_REGIONAL"/>
@@ -594,10 +605,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="contatos_teste4" displayName="contatos_teste4" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="MUNICIPIO"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="contatos_teste24" displayName="contatos_teste24" ref="A1:E39" totalsRowShown="0">
+  <autoFilter ref="A1:E39"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="MUNICIPIO_FFE"/>
+    <tableColumn id="5" name="MUNICIPIO_DL"/>
     <tableColumn id="2" name="UNIDADE_REGIONAL_FFE"/>
     <tableColumn id="3" name="EMAIL_COORDENADOR"/>
     <tableColumn id="4" name="EMAIL_UNIDADE_REGIONAL"/>
@@ -903,558 +915,676 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="54.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="C14" t="s">
         <v>49</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>50</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>51</v>
       </c>
-      <c r="D14" t="s">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" t="s">
         <v>53</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>54</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>55</v>
       </c>
-      <c r="D15" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>58</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
         <v>59</v>
       </c>
-      <c r="D16" t="s">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" t="s">
         <v>61</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
         <v>62</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
         <v>63</v>
       </c>
-      <c r="D17" t="s">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
         <v>65</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>66</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>67</v>
       </c>
-      <c r="D18" t="s">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
         <v>69</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>70</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>71</v>
       </c>
-      <c r="D19" t="s">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" t="s">
         <v>73</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>74</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
         <v>75</v>
       </c>
-      <c r="D20" t="s">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
+        <v>155</v>
+      </c>
+      <c r="C21" t="s">
         <v>77</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>78</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="1" t="s">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" t="s">
         <v>81</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
         <v>82</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>83</v>
       </c>
-      <c r="D22" t="s">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
+        <v>158</v>
+      </c>
+      <c r="C23" t="s">
         <v>85</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>86</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>87</v>
       </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
         <v>89</v>
       </c>
-      <c r="B24" t="s">
+      <c r="D24" t="s">
         <v>90</v>
       </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>91</v>
       </c>
-      <c r="D24" t="s">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" t="s">
         <v>93</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" t="s">
         <v>94</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>95</v>
       </c>
-      <c r="D25" t="s">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" t="s">
         <v>97</v>
       </c>
-      <c r="B26" t="s">
+      <c r="E26" t="s">
         <v>98</v>
       </c>
-      <c r="D26" t="s">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" t="s">
         <v>100</v>
       </c>
-      <c r="B27" t="s">
+      <c r="D27" t="s">
         <v>101</v>
       </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
         <v>102</v>
       </c>
-      <c r="D27" t="s">
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" t="s">
         <v>104</v>
       </c>
-      <c r="B28" t="s">
+      <c r="D28" t="s">
         <v>105</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E28" t="s">
         <v>106</v>
       </c>
-      <c r="D28" t="s">
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" t="s">
         <v>108</v>
       </c>
-      <c r="B29" t="s">
+      <c r="D29" t="s">
         <v>109</v>
       </c>
-      <c r="C29" t="s">
+      <c r="E29" t="s">
         <v>110</v>
       </c>
-      <c r="D29" t="s">
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" t="s">
         <v>112</v>
       </c>
-      <c r="B30" t="s">
+      <c r="D30" t="s">
         <v>113</v>
       </c>
-      <c r="C30" t="s">
+      <c r="E30" t="s">
         <v>114</v>
       </c>
-      <c r="D30" t="s">
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" t="s">
         <v>116</v>
       </c>
-      <c r="B31" t="s">
+      <c r="D31" t="s">
         <v>117</v>
       </c>
-      <c r="C31" t="s">
+      <c r="E31" t="s">
         <v>118</v>
       </c>
-      <c r="D31" t="s">
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" t="s">
         <v>120</v>
       </c>
-      <c r="B32" t="s">
+      <c r="D32" t="s">
         <v>121</v>
       </c>
-      <c r="C32" t="s">
+      <c r="E32" t="s">
         <v>122</v>
       </c>
-      <c r="D32" t="s">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" t="s">
         <v>124</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
         <v>125</v>
       </c>
-      <c r="C33" t="s">
+      <c r="E33" t="s">
         <v>126</v>
       </c>
-      <c r="D33" t="s">
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" t="s">
         <v>128</v>
       </c>
-      <c r="B34" t="s">
+      <c r="D34" t="s">
         <v>129</v>
       </c>
-      <c r="C34" t="s">
+      <c r="E34" t="s">
         <v>130</v>
       </c>
-      <c r="D34" t="s">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" t="s">
         <v>132</v>
       </c>
-      <c r="B35" t="s">
+      <c r="E35" t="s">
         <v>133</v>
       </c>
-      <c r="D35" t="s">
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" t="s">
         <v>135</v>
       </c>
-      <c r="B36" t="s">
+      <c r="D36" t="s">
         <v>136</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" t="s">
         <v>137</v>
       </c>
-      <c r="D36" t="s">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" t="s">
         <v>139</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" t="s">
         <v>140</v>
       </c>
-      <c r="C37" t="s">
+      <c r="E37" t="s">
         <v>141</v>
       </c>
-      <c r="D37" t="s">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
+        <v>142</v>
+      </c>
+      <c r="C38" t="s">
         <v>143</v>
       </c>
-      <c r="B38" t="s">
+      <c r="D38" t="s">
         <v>144</v>
       </c>
-      <c r="C38" t="s">
+      <c r="E38" t="s">
         <v>145</v>
       </c>
-      <c r="D38" t="s">
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" t="s">
         <v>147</v>
       </c>
-      <c r="B39" t="s">
+      <c r="D39" t="s">
         <v>148</v>
       </c>
-      <c r="C39" t="s">
+      <c r="E39" t="s">
         <v>149</v>
-      </c>
-      <c r="D39" t="s">
-        <v>150</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D21" r:id="rId1"/>
+    <hyperlink ref="E21" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1465,66 +1595,681 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="54.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>154</v>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" t="s">
+        <v>155</v>
+      </c>
+      <c r="C21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
+        <v>158</v>
+      </c>
+      <c r="C23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" t="s">
+        <v>97</v>
+      </c>
+      <c r="E26" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" t="s">
+        <v>101</v>
+      </c>
+      <c r="E27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" t="s">
+        <v>109</v>
+      </c>
+      <c r="E29" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" t="s">
+        <v>112</v>
+      </c>
+      <c r="D30" t="s">
+        <v>113</v>
+      </c>
+      <c r="E30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>115</v>
+      </c>
+      <c r="B31" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" t="s">
+        <v>117</v>
+      </c>
+      <c r="E31" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>119</v>
+      </c>
+      <c r="B32" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>123</v>
+      </c>
+      <c r="B33" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" t="s">
+        <v>124</v>
+      </c>
+      <c r="D33" t="s">
+        <v>125</v>
+      </c>
+      <c r="E33" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>134</v>
+      </c>
+      <c r="B36" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D36" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" t="s">
+        <v>139</v>
+      </c>
+      <c r="D37" t="s">
+        <v>140</v>
+      </c>
+      <c r="E37" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" t="s">
+        <v>142</v>
+      </c>
+      <c r="C38" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>146</v>
+      </c>
+      <c r="B39" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" t="s">
+        <v>147</v>
+      </c>
+      <c r="D39" t="s">
+        <v>148</v>
+      </c>
+      <c r="E39" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
+    <hyperlink ref="E21" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>